<commit_message>
Refine image grading and paper limitations
</commit_message>
<xml_diff>
--- a/paper/tables/main_tables.xlsx
+++ b/paper/tables/main_tables.xlsx
@@ -12,8 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标矩阵" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="组合权重" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图像评分" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视频时序" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数审计" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="相对等级" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视频时序" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数审计" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -822,7 +823,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
   </cols>
@@ -857,7 +858,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>语义要素覆盖代理</t>
+          <t>语义结构完整性代理</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -1872,7 +1873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1882,8 +1883,13 @@
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1924,10 +1930,35 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
+          <t>absolute_quality_grade</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>relative_quality_tier</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>key_strength</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>key_weakness</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
           <t>final_grade</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>semantic_final_grade</t>
         </is>
@@ -1968,6 +1999,29 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
+          <t>相对中</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>视觉表达</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>中等</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
           <t>中等</t>
         </is>
       </c>
@@ -2007,6 +2061,29 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
+          <t>相对中</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>结构完整性</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>中等</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
           <t>中等</t>
         </is>
       </c>
@@ -2046,6 +2123,29 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
+          <t>相对低</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>结构完整性</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>较低</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
           <t>较低</t>
         </is>
       </c>
@@ -2085,6 +2185,29 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
+          <t>相对高</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>结构完整性</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>中等</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
           <t>中等</t>
         </is>
       </c>
@@ -2124,6 +2247,29 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
+          <t>相对高</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>视觉表达</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>中等</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
           <t>中等</t>
         </is>
       </c>
@@ -2163,6 +2309,29 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
+          <t>相对中</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>视觉表达</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>中等</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
           <t>中等</t>
         </is>
       </c>
@@ -2202,6 +2371,29 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
+          <t>相对低</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>视觉表达</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>较低</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
           <t>较低</t>
         </is>
       </c>
@@ -2240,6 +2432,29 @@
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>相对低</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>语义结构完整性代理</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>较低</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
         <is>
           <t>较低</t>
         </is>
@@ -2251,6 +2466,422 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>sample_id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>content_type</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Q_final</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>absolute_quality_grade</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>relative_quality_tier</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>key_strength</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>key_weakness</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>image_05</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>5.jpg</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>写实风景</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>62.22703934587288</v>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>中等</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>相对高</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>视觉表达</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>image_04</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>4.png</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>动态街景</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>59.3413781906943</v>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>中等</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>相对高</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>结构完整性</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>image_02</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>2.png</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>人物肖像</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>58.20052770030814</v>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>中等</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>相对中</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>结构完整性</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>image_01</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>1.png</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>写实风景</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>57.67818232498608</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>中等</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>相对中</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>视觉表达</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>image_06</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>6.jpg</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>人物插画</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>55.22183896321834</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>中等</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>相对中</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>视觉表达</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>image_08</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>8.jpg</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>像素街景</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>53.41153482967204</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>较低</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>相对低</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>语义结构完整性代理</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>image_07</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>7.jpg</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>水墨插画</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>52.5004842483709</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>较低</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>相对低</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>视觉表达</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>image_03</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>3.png</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>艺术插画</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>42.41033674000774</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>较低</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>相对低</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>伪影抑制</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>结构完整性</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2436,7 +3067,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>